<commit_message>
se agrego nuevo campo de fecha para guardar en excel de errores
</commit_message>
<xml_diff>
--- a/app/Templates/plantilla_errores.xlsx
+++ b/app/Templates/plantilla_errores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">ID FACTURA</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL EN BD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA DE PAGO</t>
   </si>
 </sst>
 </file>
@@ -119,7 +122,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -129,6 +132,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -255,7 +262,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.58"/>
@@ -264,6 +271,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.07"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -284,6 +292,9 @@
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>